<commit_message>
Cleaning for Zenodo update
</commit_message>
<xml_diff>
--- a/data/Mappings/mapping_ctrace.xlsx
+++ b/data/Mappings/mapping_ctrace.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca0-my.sharepoint.com/personal/marin_pellan_polymtlus_ca/Documents/Desktop/POST_DOC/Project/canada_metal_sustainability_db/data/Mappings/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/metallican_db/data/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F080618-ACD9-4DD8-8E4A-561DAF1AAAA3}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{039DCBCC-66E5-4413-96AE-BDDDFD54A0CC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LT" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">LT!$A$1:$G$318</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">mapping!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="602">
   <si>
     <t>main_id</t>
   </si>
@@ -1876,10 +1877,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1895,6 +1895,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2161,18 +2165,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G318"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2195,7 +2199,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -2218,7 +2222,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -2241,7 +2245,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -2264,7 +2268,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -2287,7 +2291,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
@@ -2310,7 +2314,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
@@ -2333,7 +2337,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
@@ -2356,7 +2360,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -2379,7 +2383,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>31</v>
       </c>
@@ -2402,7 +2406,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
@@ -2425,7 +2429,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>37</v>
       </c>
@@ -2448,7 +2452,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>40</v>
       </c>
@@ -2471,7 +2475,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>43</v>
       </c>
@@ -2494,7 +2498,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>46</v>
       </c>
@@ -2517,7 +2521,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>49</v>
       </c>
@@ -2540,7 +2544,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>52</v>
       </c>
@@ -2563,7 +2567,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>55</v>
       </c>
@@ -2586,7 +2590,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>57</v>
       </c>
@@ -2609,7 +2613,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>60</v>
       </c>
@@ -2632,7 +2636,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>63</v>
       </c>
@@ -2655,7 +2659,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>66</v>
       </c>
@@ -2678,7 +2682,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>69</v>
       </c>
@@ -2701,7 +2705,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>72</v>
       </c>
@@ -2724,7 +2728,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>75</v>
       </c>
@@ -2747,7 +2751,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>78</v>
       </c>
@@ -2770,7 +2774,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>81</v>
       </c>
@@ -2793,7 +2797,7 @@
         <v>82.758620689655103</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -2816,7 +2820,7 @@
         <v>82.758620689655103</v>
       </c>
     </row>
-    <row r="29" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>85</v>
       </c>
@@ -2839,7 +2843,7 @@
         <v>76.190476190476105</v>
       </c>
     </row>
-    <row r="30" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>88</v>
       </c>
@@ -2862,7 +2866,7 @@
         <v>75.862068965517196</v>
       </c>
     </row>
-    <row r="31" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>91</v>
       </c>
@@ -2885,7 +2889,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>94</v>
       </c>
@@ -2908,7 +2912,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>96</v>
       </c>
@@ -2931,7 +2935,7 @@
         <v>36.363636363636303</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>98</v>
       </c>
@@ -2954,7 +2958,7 @@
         <v>34.782608695652101</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>100</v>
       </c>
@@ -2977,7 +2981,7 @@
         <v>33.3333333333333</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>103</v>
       </c>
@@ -3000,7 +3004,7 @@
         <v>33.3333333333333</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>105</v>
       </c>
@@ -3023,7 +3027,7 @@
         <v>32.4324324324324</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>81</v>
       </c>
@@ -3046,7 +3050,7 @@
         <v>32.258064516128997</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>84</v>
       </c>
@@ -3069,7 +3073,7 @@
         <v>32.258064516128997</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>108</v>
       </c>
@@ -3092,7 +3096,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -3115,7 +3119,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>110</v>
       </c>
@@ -3138,7 +3142,7 @@
         <v>30.769230769230699</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>72</v>
       </c>
@@ -3161,7 +3165,7 @@
         <v>30.769230769230699</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>113</v>
       </c>
@@ -3184,7 +3188,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>72</v>
       </c>
@@ -3207,7 +3211,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>103</v>
       </c>
@@ -3230,7 +3234,7 @@
         <v>29.629629629629601</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>81</v>
       </c>
@@ -3253,7 +3257,7 @@
         <v>29.411764705882302</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>84</v>
       </c>
@@ -3276,7 +3280,7 @@
         <v>29.411764705882302</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>115</v>
       </c>
@@ -3299,7 +3303,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>103</v>
       </c>
@@ -3322,7 +3326,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>117</v>
       </c>
@@ -3345,7 +3349,7 @@
         <v>27.586206896551701</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>117</v>
       </c>
@@ -3368,7 +3372,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>121</v>
       </c>
@@ -3391,7 +3395,7 @@
         <v>26.086956521739101</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>108</v>
       </c>
@@ -3414,7 +3418,7 @@
         <v>25.806451612903199</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>69</v>
       </c>
@@ -3437,7 +3441,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>19</v>
       </c>
@@ -3460,7 +3464,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>124</v>
       </c>
@@ -3483,7 +3487,7 @@
         <v>23.076923076922998</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>117</v>
       </c>
@@ -3506,7 +3510,7 @@
         <v>23.076923076922998</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>127</v>
       </c>
@@ -3529,7 +3533,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>117</v>
       </c>
@@ -3552,7 +3556,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>117</v>
       </c>
@@ -3575,7 +3579,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>75</v>
       </c>
@@ -3598,7 +3602,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>96</v>
       </c>
@@ -3621,7 +3625,7 @@
         <v>21.052631578947299</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>25</v>
       </c>
@@ -3644,7 +3648,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>81</v>
       </c>
@@ -3667,7 +3671,7 @@
         <v>19.354838709677399</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>84</v>
       </c>
@@ -3690,7 +3694,7 @@
         <v>19.354838709677399</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>94</v>
       </c>
@@ -3713,7 +3717,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>103</v>
       </c>
@@ -3736,7 +3740,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>132</v>
       </c>
@@ -3759,7 +3763,7 @@
         <v>18.181818181818102</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>75</v>
       </c>
@@ -3782,7 +3786,7 @@
         <v>17.391304347826001</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>127</v>
       </c>
@@ -3805,7 +3809,7 @@
         <v>16.6666666666666</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>117</v>
       </c>
@@ -3828,7 +3832,7 @@
         <v>16.6666666666666</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>135</v>
       </c>
@@ -3851,7 +3855,7 @@
         <v>15.3846153846153</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>105</v>
       </c>
@@ -3874,7 +3878,7 @@
         <v>14.814814814814801</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>100</v>
       </c>
@@ -3897,7 +3901,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>132</v>
       </c>
@@ -3920,7 +3924,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>75</v>
       </c>
@@ -3943,7 +3947,7 @@
         <v>11.764705882352899</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>28</v>
       </c>
@@ -3966,7 +3970,7 @@
         <v>11.1111111111111</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>138</v>
       </c>
@@ -3989,7 +3993,7 @@
         <v>9.5238095238095095</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>140</v>
       </c>
@@ -4012,7 +4016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>141</v>
       </c>
@@ -4035,7 +4039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>144</v>
       </c>
@@ -4043,7 +4047,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>146</v>
       </c>
@@ -4051,7 +4055,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>148</v>
       </c>
@@ -4059,7 +4063,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>150</v>
       </c>
@@ -4067,7 +4071,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>152</v>
       </c>
@@ -4075,7 +4079,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>154</v>
       </c>
@@ -4083,7 +4087,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>156</v>
       </c>
@@ -4091,7 +4095,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>158</v>
       </c>
@@ -4099,7 +4103,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>160</v>
       </c>
@@ -4107,7 +4111,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>162</v>
       </c>
@@ -4115,7 +4119,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>164</v>
       </c>
@@ -4123,7 +4127,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>166</v>
       </c>
@@ -4131,7 +4135,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>168</v>
       </c>
@@ -4139,7 +4143,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>170</v>
       </c>
@@ -4147,7 +4151,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>172</v>
       </c>
@@ -4155,7 +4159,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>174</v>
       </c>
@@ -4163,7 +4167,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>176</v>
       </c>
@@ -4171,7 +4175,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>178</v>
       </c>
@@ -4179,7 +4183,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>180</v>
       </c>
@@ -4187,7 +4191,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>182</v>
       </c>
@@ -4195,7 +4199,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>184</v>
       </c>
@@ -4203,7 +4207,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>186</v>
       </c>
@@ -4211,7 +4215,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>188</v>
       </c>
@@ -4219,7 +4223,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>190</v>
       </c>
@@ -4227,7 +4231,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>192</v>
       </c>
@@ -4235,7 +4239,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>194</v>
       </c>
@@ -4243,7 +4247,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>196</v>
       </c>
@@ -4251,7 +4255,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>198</v>
       </c>
@@ -4259,7 +4263,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>200</v>
       </c>
@@ -4267,7 +4271,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>202</v>
       </c>
@@ -4275,7 +4279,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>204</v>
       </c>
@@ -4283,7 +4287,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>206</v>
       </c>
@@ -4291,7 +4295,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>208</v>
       </c>
@@ -4299,7 +4303,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>210</v>
       </c>
@@ -4307,7 +4311,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>212</v>
       </c>
@@ -4315,7 +4319,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>214</v>
       </c>
@@ -4323,7 +4327,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>216</v>
       </c>
@@ -4331,7 +4335,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>218</v>
       </c>
@@ -4339,7 +4343,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>220</v>
       </c>
@@ -4347,7 +4351,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>222</v>
       </c>
@@ -4355,7 +4359,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>224</v>
       </c>
@@ -4363,7 +4367,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>226</v>
       </c>
@@ -4371,7 +4375,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>228</v>
       </c>
@@ -4379,7 +4383,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>230</v>
       </c>
@@ -4387,7 +4391,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>232</v>
       </c>
@@ -4395,7 +4399,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>234</v>
       </c>
@@ -4403,7 +4407,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>236</v>
       </c>
@@ -4411,7 +4415,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>238</v>
       </c>
@@ -4419,7 +4423,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>240</v>
       </c>
@@ -4427,7 +4431,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>242</v>
       </c>
@@ -4435,7 +4439,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>244</v>
       </c>
@@ -4443,7 +4447,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>246</v>
       </c>
@@ -4451,7 +4455,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>248</v>
       </c>
@@ -4459,7 +4463,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>250</v>
       </c>
@@ -4467,7 +4471,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>252</v>
       </c>
@@ -4475,7 +4479,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>254</v>
       </c>
@@ -4483,7 +4487,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>256</v>
       </c>
@@ -4491,7 +4495,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>258</v>
       </c>
@@ -4499,7 +4503,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>260</v>
       </c>
@@ -4507,7 +4511,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>262</v>
       </c>
@@ -4515,7 +4519,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>264</v>
       </c>
@@ -4523,7 +4527,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>266</v>
       </c>
@@ -4531,7 +4535,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>268</v>
       </c>
@@ -4539,7 +4543,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>270</v>
       </c>
@@ -4547,7 +4551,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>272</v>
       </c>
@@ -4555,7 +4559,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>274</v>
       </c>
@@ -4563,7 +4567,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>276</v>
       </c>
@@ -4571,7 +4575,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>278</v>
       </c>
@@ -4579,7 +4583,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>280</v>
       </c>
@@ -4587,7 +4591,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>282</v>
       </c>
@@ -4595,7 +4599,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>284</v>
       </c>
@@ -4603,7 +4607,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>286</v>
       </c>
@@ -4611,7 +4615,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>288</v>
       </c>
@@ -4619,7 +4623,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>290</v>
       </c>
@@ -4627,7 +4631,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>292</v>
       </c>
@@ -4635,7 +4639,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>294</v>
       </c>
@@ -4643,7 +4647,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>296</v>
       </c>
@@ -4651,7 +4655,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>298</v>
       </c>
@@ -4659,7 +4663,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>300</v>
       </c>
@@ -4667,7 +4671,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>302</v>
       </c>
@@ -4675,7 +4679,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>304</v>
       </c>
@@ -4683,7 +4687,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>306</v>
       </c>
@@ -4691,7 +4695,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>308</v>
       </c>
@@ -4699,7 +4703,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>310</v>
       </c>
@@ -4707,7 +4711,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>312</v>
       </c>
@@ -4715,7 +4719,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>314</v>
       </c>
@@ -4723,7 +4727,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>316</v>
       </c>
@@ -4731,7 +4735,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>318</v>
       </c>
@@ -4739,7 +4743,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>320</v>
       </c>
@@ -4747,7 +4751,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>322</v>
       </c>
@@ -4755,7 +4759,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>324</v>
       </c>
@@ -4763,7 +4767,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>326</v>
       </c>
@@ -4771,7 +4775,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>328</v>
       </c>
@@ -4779,7 +4783,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>330</v>
       </c>
@@ -4787,7 +4791,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>332</v>
       </c>
@@ -4795,7 +4799,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>334</v>
       </c>
@@ -4803,7 +4807,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>336</v>
       </c>
@@ -4811,7 +4815,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>338</v>
       </c>
@@ -4819,7 +4823,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>340</v>
       </c>
@@ -4827,7 +4831,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>342</v>
       </c>
@@ -4835,7 +4839,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>344</v>
       </c>
@@ -4843,7 +4847,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>346</v>
       </c>
@@ -4851,7 +4855,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>348</v>
       </c>
@@ -4859,7 +4863,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>350</v>
       </c>
@@ -4867,7 +4871,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>352</v>
       </c>
@@ -4875,7 +4879,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>354</v>
       </c>
@@ -4883,7 +4887,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>356</v>
       </c>
@@ -4891,7 +4895,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>358</v>
       </c>
@@ -4899,7 +4903,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>360</v>
       </c>
@@ -4907,7 +4911,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>362</v>
       </c>
@@ -4915,7 +4919,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>364</v>
       </c>
@@ -4923,7 +4927,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>366</v>
       </c>
@@ -4931,7 +4935,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>368</v>
       </c>
@@ -4939,7 +4943,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>370</v>
       </c>
@@ -4947,7 +4951,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>372</v>
       </c>
@@ -4955,7 +4959,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>374</v>
       </c>
@@ -4963,7 +4967,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>376</v>
       </c>
@@ -4971,7 +4975,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>378</v>
       </c>
@@ -4979,7 +4983,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>380</v>
       </c>
@@ -4987,7 +4991,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>382</v>
       </c>
@@ -4995,7 +4999,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>384</v>
       </c>
@@ -5003,7 +5007,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>386</v>
       </c>
@@ -5011,7 +5015,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>388</v>
       </c>
@@ -5019,7 +5023,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>390</v>
       </c>
@@ -5027,7 +5031,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>392</v>
       </c>
@@ -5035,7 +5039,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>394</v>
       </c>
@@ -5043,7 +5047,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>396</v>
       </c>
@@ -5051,7 +5055,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>398</v>
       </c>
@@ -5059,7 +5063,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>400</v>
       </c>
@@ -5067,7 +5071,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>402</v>
       </c>
@@ -5075,7 +5079,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>404</v>
       </c>
@@ -5083,7 +5087,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>406</v>
       </c>
@@ -5091,7 +5095,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>408</v>
       </c>
@@ -5099,7 +5103,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>410</v>
       </c>
@@ -5107,7 +5111,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>412</v>
       </c>
@@ -5115,7 +5119,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>414</v>
       </c>
@@ -5123,7 +5127,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>416</v>
       </c>
@@ -5131,7 +5135,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>418</v>
       </c>
@@ -5139,7 +5143,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>420</v>
       </c>
@@ -5147,7 +5151,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>422</v>
       </c>
@@ -5155,7 +5159,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>424</v>
       </c>
@@ -5163,7 +5167,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>426</v>
       </c>
@@ -5171,7 +5175,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>428</v>
       </c>
@@ -5179,7 +5183,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>430</v>
       </c>
@@ -5187,7 +5191,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>432</v>
       </c>
@@ -5195,7 +5199,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>434</v>
       </c>
@@ -5203,7 +5207,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>436</v>
       </c>
@@ -5211,7 +5215,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>438</v>
       </c>
@@ -5219,7 +5223,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>440</v>
       </c>
@@ -5227,7 +5231,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>442</v>
       </c>
@@ -5235,7 +5239,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>444</v>
       </c>
@@ -5243,7 +5247,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>446</v>
       </c>
@@ -5251,7 +5255,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>448</v>
       </c>
@@ -5259,7 +5263,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>450</v>
       </c>
@@ -5267,7 +5271,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>452</v>
       </c>
@@ -5275,7 +5279,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>454</v>
       </c>
@@ -5283,7 +5287,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>456</v>
       </c>
@@ -5291,7 +5295,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>458</v>
       </c>
@@ -5299,7 +5303,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>460</v>
       </c>
@@ -5307,7 +5311,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>462</v>
       </c>
@@ -5315,7 +5319,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>464</v>
       </c>
@@ -5323,7 +5327,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>466</v>
       </c>
@@ -5331,7 +5335,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>468</v>
       </c>
@@ -5339,7 +5343,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>470</v>
       </c>
@@ -5347,7 +5351,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>472</v>
       </c>
@@ -5355,7 +5359,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>474</v>
       </c>
@@ -5363,7 +5367,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>476</v>
       </c>
@@ -5371,7 +5375,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>478</v>
       </c>
@@ -5379,7 +5383,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>480</v>
       </c>
@@ -5387,7 +5391,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>482</v>
       </c>
@@ -5395,7 +5399,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>484</v>
       </c>
@@ -5403,7 +5407,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>486</v>
       </c>
@@ -5411,7 +5415,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>488</v>
       </c>
@@ -5419,7 +5423,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>490</v>
       </c>
@@ -5427,7 +5431,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>492</v>
       </c>
@@ -5435,7 +5439,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>494</v>
       </c>
@@ -5443,7 +5447,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>496</v>
       </c>
@@ -5451,7 +5455,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>498</v>
       </c>
@@ -5459,7 +5463,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>500</v>
       </c>
@@ -5467,7 +5471,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>502</v>
       </c>
@@ -5475,7 +5479,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>504</v>
       </c>
@@ -5483,7 +5487,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>506</v>
       </c>
@@ -5491,7 +5495,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>508</v>
       </c>
@@ -5499,7 +5503,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>510</v>
       </c>
@@ -5507,7 +5511,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>512</v>
       </c>
@@ -5515,7 +5519,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>514</v>
       </c>
@@ -5523,7 +5527,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>516</v>
       </c>
@@ -5531,7 +5535,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>518</v>
       </c>
@@ -5539,7 +5543,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>520</v>
       </c>
@@ -5547,7 +5551,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>522</v>
       </c>
@@ -5555,7 +5559,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>524</v>
       </c>
@@ -5563,7 +5567,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>526</v>
       </c>
@@ -5571,7 +5575,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>528</v>
       </c>
@@ -5579,7 +5583,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>530</v>
       </c>
@@ -5587,7 +5591,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>532</v>
       </c>
@@ -5595,7 +5599,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>534</v>
       </c>
@@ -5603,7 +5607,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>536</v>
       </c>
@@ -5611,7 +5615,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>538</v>
       </c>
@@ -5619,7 +5623,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>540</v>
       </c>
@@ -5627,7 +5631,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>542</v>
       </c>
@@ -5635,7 +5639,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>544</v>
       </c>
@@ -5643,7 +5647,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="283" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>546</v>
       </c>
@@ -5651,7 +5655,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="284" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>548</v>
       </c>
@@ -5659,7 +5663,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="285" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>550</v>
       </c>
@@ -5667,7 +5671,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="286" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>552</v>
       </c>
@@ -5675,7 +5679,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="287" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>554</v>
       </c>
@@ -5683,7 +5687,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="288" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>556</v>
       </c>
@@ -5691,7 +5695,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>558</v>
       </c>
@@ -5699,7 +5703,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>560</v>
       </c>
@@ -5707,7 +5711,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>562</v>
       </c>
@@ -5715,7 +5719,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>564</v>
       </c>
@@ -5723,7 +5727,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>566</v>
       </c>
@@ -5731,7 +5735,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>568</v>
       </c>
@@ -5739,7 +5743,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>570</v>
       </c>
@@ -5747,7 +5751,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>572</v>
       </c>
@@ -5755,7 +5759,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>574</v>
       </c>
@@ -5763,7 +5767,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>576</v>
       </c>
@@ -5771,7 +5775,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>578</v>
       </c>
@@ -5779,7 +5783,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>580</v>
       </c>
@@ -5787,7 +5791,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>582</v>
       </c>
@@ -5795,7 +5799,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>584</v>
       </c>
@@ -5803,7 +5807,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B303">
         <v>1754048</v>
       </c>
@@ -5811,7 +5815,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B304">
         <v>1754049</v>
       </c>
@@ -5819,7 +5823,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="305" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="305" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B305">
         <v>1754051</v>
       </c>
@@ -5827,7 +5831,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="306" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="306" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B306">
         <v>1754053</v>
       </c>
@@ -5835,7 +5839,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="307" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="307" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B307">
         <v>1754059</v>
       </c>
@@ -5843,7 +5847,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="308" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="308" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B308">
         <v>1754063</v>
       </c>
@@ -5851,7 +5855,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="309" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="309" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B309">
         <v>1754064</v>
       </c>
@@ -5859,7 +5863,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="310" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="310" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B310">
         <v>1754065</v>
       </c>
@@ -5867,7 +5871,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="311" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="311" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B311">
         <v>1754070</v>
       </c>
@@ -5875,7 +5879,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="312" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="312" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B312">
         <v>1754076</v>
       </c>
@@ -5883,7 +5887,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="313" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="313" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B313">
         <v>1754080</v>
       </c>
@@ -5891,7 +5895,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="314" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="314" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B314">
         <v>1754089</v>
       </c>
@@ -5899,7 +5903,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="315" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="315" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B315">
         <v>1754093</v>
       </c>
@@ -5907,7 +5911,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="316" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="316" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B316">
         <v>1754095</v>
       </c>
@@ -5915,7 +5919,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="317" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="317" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B317">
         <v>1754099</v>
       </c>
@@ -5923,7 +5927,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="318" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="318" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B318">
         <v>1754100</v>
       </c>
@@ -5939,10 +5943,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40E14CAD-8146-48AD-B241-383098A7250B}">
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -5950,239 +5958,236 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1754055</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1754056</v>
+      </c>
+      <c r="B3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>1754057</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>1754058</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>1754060</v>
+      </c>
+      <c r="B6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1754061</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1754066</v>
+      </c>
+      <c r="B8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1754067</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>1754071</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1754075</v>
+      </c>
+      <c r="B11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12">
         <v>1754077</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>1754071</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1754081</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>1754082</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1754083</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16">
         <v>1754084</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>1754082</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>1754067</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1754085</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>1754086</v>
+      </c>
+      <c r="B18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1754087</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>1754096</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>1754097</v>
+      </c>
+      <c r="B21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>1754102</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>1754103</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>1754104</v>
+      </c>
+      <c r="B24" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>1754105</v>
+      </c>
+      <c r="B25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>1754106</v>
+      </c>
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27">
         <v>25486533</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B27" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
-        <v>1754096</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>1754102</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
-        <v>1754057</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28">
         <v>25486534</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>1754085</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
-        <v>1754081</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
-        <v>1754083</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
-        <v>1754087</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
-        <v>1754097</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29">
         <v>36395102</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B29" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
-        <v>36395102</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
-        <v>1754061</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2">
-        <v>1754066</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
-        <v>1754086</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
-        <v>1754105</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="2">
-        <v>1754055</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
-        <v>1754058</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="2">
-        <v>1754060</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>1754104</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
-        <v>1754056</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="2">
-        <v>1754103</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2">
-        <v>1754106</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>1754075</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:B1" xr:uid="{40E14CAD-8146-48AD-B241-383098A7250B}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B29">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>